<commit_message>
add pivot table calculation
</commit_message>
<xml_diff>
--- a/model.xlsx
+++ b/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\world\Desktop\macros\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C2353D81-7BFE-4F32-A8D4-C6FD1B6CAEA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB15CAB7-798F-41BC-A1F7-C44EAF547C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Расчётная модель SIP" sheetId="1" r:id="rId1"/>
@@ -249,7 +249,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="817" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="936" uniqueCount="73">
   <si>
     <t>Q1</t>
   </si>
@@ -477,7 +477,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="28" x14ac:knownFonts="1">
+  <fonts count="27" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -644,13 +644,6 @@
       <b/>
       <sz val="12"/>
       <color rgb="FFFF0000"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1421,7 +1414,7 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="182">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1740,12 +1733,6 @@
     <xf numFmtId="9" fontId="9" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="10" fontId="8" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1762,9 +1749,6 @@
     <xf numFmtId="164" fontId="23" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="45" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="21" xfId="0" applyBorder="1"/>
     <xf numFmtId="10" fontId="9" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1773,12 +1757,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="9" fontId="9" fillId="0" borderId="41" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="40" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1802,20 +1780,11 @@
     <xf numFmtId="164" fontId="20" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="9" fontId="24" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="24" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="9" fontId="19" fillId="0" borderId="17" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="48" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="17" fillId="0" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1824,10 +1793,10 @@
     <xf numFmtId="164" fontId="17" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="10" fontId="26" fillId="0" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="25" fillId="0" borderId="49" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="26" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="25" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="18" fillId="0" borderId="51" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1836,7 +1805,7 @@
     <xf numFmtId="164" fontId="18" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="27" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="26" fillId="0" borderId="50" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -3769,7 +3738,7 @@
     <row r="15" spans="1:43" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:43" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43"/>
-      <c r="B16" s="155" t="s">
+      <c r="B16" s="147" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="44" t="s">
@@ -4499,7 +4468,7 @@
         <v>0.28500000000000003</v>
       </c>
       <c r="G23" s="73">
-        <f t="shared" si="30"/>
+        <f>SUM(G17:G22)</f>
         <v>0.27784615384615385</v>
       </c>
       <c r="H23" s="73">
@@ -4663,7 +4632,7 @@
     </row>
     <row r="25" spans="1:35" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43"/>
-      <c r="B25" s="155"/>
+      <c r="B25" s="147"/>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
@@ -5323,8 +5292,8 @@
       </c>
     </row>
     <row r="34" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="C34" s="162"/>
-      <c r="D34" s="162"/>
+      <c r="C34" s="154"/>
+      <c r="D34" s="154"/>
       <c r="L34" s="31">
         <f t="shared" si="41"/>
         <v>281.80855199999996</v>
@@ -10095,10 +10064,10 @@
         <f t="shared" ref="L41:L56" si="3">F41/E41</f>
         <v>0.99424811189673923</v>
       </c>
-      <c r="M41" s="172">
+      <c r="M41" s="164">
         <v>1.0449999999999999</v>
       </c>
-      <c r="O41" s="168"/>
+      <c r="O41" s="160"/>
     </row>
     <row r="42" spans="1:15" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A42">
@@ -10427,7 +10396,7 @@
         <v>1.0022481051974976</v>
       </c>
       <c r="M49" s="23"/>
-      <c r="O49" s="168"/>
+      <c r="O49" s="160"/>
     </row>
     <row r="50" spans="1:20" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A50">
@@ -10509,7 +10478,7 @@
         <f t="shared" si="3"/>
         <v>0.99739977865224694</v>
       </c>
-      <c r="M51" s="172">
+      <c r="M51" s="164">
         <v>1.034</v>
       </c>
     </row>
@@ -10786,7 +10755,7 @@
       <c r="S59" s="23" t="s">
         <v>72</v>
       </c>
-      <c r="T59" s="171"/>
+      <c r="T59" s="163"/>
     </row>
     <row r="60" spans="1:20" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60">
@@ -10830,8 +10799,8 @@
       <c r="M60" s="90"/>
       <c r="O60" s="91"/>
       <c r="P60" s="90"/>
-      <c r="R60" s="169"/>
-      <c r="S60" s="172">
+      <c r="R60" s="161"/>
+      <c r="S60" s="164">
         <v>1.0449999999999999</v>
       </c>
       <c r="T60" s="13"/>
@@ -10878,7 +10847,7 @@
       <c r="M61" s="90"/>
       <c r="O61" s="91"/>
       <c r="P61" s="90"/>
-      <c r="R61" s="169"/>
+      <c r="R61" s="161"/>
       <c r="S61" s="23"/>
       <c r="T61" s="13"/>
     </row>
@@ -10924,7 +10893,7 @@
       <c r="M62" s="90"/>
       <c r="O62" s="91"/>
       <c r="P62" s="90"/>
-      <c r="R62" s="169"/>
+      <c r="R62" s="161"/>
       <c r="S62" s="23"/>
       <c r="T62" s="13"/>
     </row>
@@ -10970,7 +10939,7 @@
       <c r="M63" s="90"/>
       <c r="O63" s="91"/>
       <c r="P63" s="90"/>
-      <c r="R63" s="169"/>
+      <c r="R63" s="161"/>
       <c r="S63" s="23"/>
       <c r="T63" s="13"/>
     </row>
@@ -11016,7 +10985,7 @@
       <c r="M64" s="90"/>
       <c r="O64" s="91"/>
       <c r="P64" s="90"/>
-      <c r="R64" s="169"/>
+      <c r="R64" s="161"/>
       <c r="S64" s="23"/>
       <c r="T64" s="13"/>
     </row>
@@ -11062,7 +11031,7 @@
       <c r="M65" s="90"/>
       <c r="O65" s="91"/>
       <c r="P65" s="90"/>
-      <c r="R65" s="169"/>
+      <c r="R65" s="161"/>
       <c r="S65" s="23"/>
       <c r="T65" s="13"/>
     </row>
@@ -11108,7 +11077,7 @@
       <c r="M66" s="90"/>
       <c r="O66" s="91"/>
       <c r="P66" s="90"/>
-      <c r="R66" s="169"/>
+      <c r="R66" s="161"/>
       <c r="S66" s="23"/>
       <c r="T66" s="13"/>
     </row>
@@ -11154,7 +11123,7 @@
       <c r="M67" s="90"/>
       <c r="O67" s="91"/>
       <c r="P67" s="90"/>
-      <c r="R67" s="169"/>
+      <c r="R67" s="161"/>
       <c r="S67" s="23"/>
       <c r="T67" s="13"/>
     </row>
@@ -11200,7 +11169,7 @@
       <c r="M68" s="90"/>
       <c r="O68" s="91"/>
       <c r="P68" s="90"/>
-      <c r="R68" s="169"/>
+      <c r="R68" s="161"/>
       <c r="S68" s="23"/>
       <c r="T68" s="13"/>
     </row>
@@ -11246,7 +11215,7 @@
       <c r="M69" s="90"/>
       <c r="O69" s="91"/>
       <c r="P69" s="90"/>
-      <c r="R69" s="169"/>
+      <c r="R69" s="161"/>
       <c r="S69" s="23"/>
       <c r="T69" s="13"/>
     </row>
@@ -11305,11 +11274,11 @@
       <c r="Q70" s="106">
         <v>40933</v>
       </c>
-      <c r="R70" s="170">
+      <c r="R70" s="162">
         <f>Q70/P70</f>
         <v>1.0122159301664235</v>
       </c>
-      <c r="S70" s="172">
+      <c r="S70" s="164">
         <v>1.034</v>
       </c>
       <c r="T70" s="1"/>
@@ -11356,7 +11325,7 @@
       <c r="M71" s="90"/>
       <c r="O71" s="91"/>
       <c r="P71" s="90"/>
-      <c r="R71" s="169"/>
+      <c r="R71" s="161"/>
       <c r="S71" s="23"/>
       <c r="T71" s="13"/>
     </row>
@@ -11402,7 +11371,7 @@
       <c r="M72" s="90"/>
       <c r="O72" s="91"/>
       <c r="P72" s="90"/>
-      <c r="R72" s="169"/>
+      <c r="R72" s="161"/>
       <c r="S72" s="23"/>
       <c r="T72" s="13"/>
     </row>
@@ -11448,7 +11417,7 @@
       <c r="M73" s="90"/>
       <c r="O73" s="91"/>
       <c r="P73" s="90"/>
-      <c r="R73" s="169"/>
+      <c r="R73" s="161"/>
       <c r="S73" s="23"/>
       <c r="T73" s="13"/>
     </row>
@@ -11494,7 +11463,7 @@
       <c r="M74" s="90"/>
       <c r="O74" s="91"/>
       <c r="P74" s="90"/>
-      <c r="R74" s="169"/>
+      <c r="R74" s="161"/>
       <c r="S74" s="23"/>
       <c r="T74" s="13"/>
     </row>
@@ -11561,71 +11530,76 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="B1:Q20"/>
+  <dimension ref="B1:AJ86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="12.85546875" customWidth="1"/>
-    <col min="4" max="17" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="17" width="11.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="2" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="2:36" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:36" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
-      <c r="D2" s="180" t="s">
+      <c r="D2" s="172" t="s">
         <v>62</v>
       </c>
-      <c r="E2" s="181"/>
-      <c r="F2" s="181"/>
-      <c r="G2" s="181"/>
-      <c r="H2" s="181"/>
-      <c r="I2" s="182"/>
-      <c r="J2" s="180" t="s">
+      <c r="E2" s="173"/>
+      <c r="F2" s="173"/>
+      <c r="G2" s="173"/>
+      <c r="H2" s="173"/>
+      <c r="I2" s="174"/>
+      <c r="J2" s="172" t="s">
         <v>63</v>
       </c>
-      <c r="K2" s="181"/>
-      <c r="L2" s="181"/>
-      <c r="M2" s="181"/>
-      <c r="N2" s="181"/>
-      <c r="O2" s="181"/>
-      <c r="P2" s="181"/>
-      <c r="Q2" s="182"/>
-    </row>
-    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
-      <c r="C3" s="179" t="s">
+      <c r="K2" s="173"/>
+      <c r="L2" s="173"/>
+      <c r="M2" s="173"/>
+      <c r="N2" s="173"/>
+      <c r="O2" s="173"/>
+      <c r="P2" s="173"/>
+      <c r="Q2" s="174"/>
+    </row>
+    <row r="3" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="C3" s="171" t="s">
         <v>64</v>
       </c>
-      <c r="D3" s="173" t="s">
+      <c r="D3" s="165" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="174"/>
-      <c r="F3" s="173" t="s">
+      <c r="E3" s="166"/>
+      <c r="F3" s="165" t="s">
         <v>25</v>
       </c>
-      <c r="G3" s="174"/>
-      <c r="H3" s="189">
+      <c r="G3" s="166"/>
+      <c r="H3" s="181">
         <v>1</v>
       </c>
-      <c r="I3" s="174"/>
-      <c r="J3" s="173" t="s">
+      <c r="I3" s="166"/>
+      <c r="J3" s="165" t="s">
         <v>65</v>
       </c>
-      <c r="K3" s="174"/>
-      <c r="L3" s="173" t="s">
+      <c r="K3" s="166"/>
+      <c r="L3" s="165" t="s">
         <v>25</v>
       </c>
-      <c r="M3" s="174"/>
-      <c r="N3" s="173" t="s">
+      <c r="M3" s="166"/>
+      <c r="N3" s="165" t="s">
         <v>66</v>
       </c>
-      <c r="O3" s="174"/>
-      <c r="P3" s="175" t="s">
+      <c r="O3" s="166"/>
+      <c r="P3" s="167" t="s">
         <v>24</v>
       </c>
-      <c r="Q3" s="174"/>
-    </row>
-    <row r="4" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="C4" s="178"/>
+      <c r="Q3" s="166"/>
+    </row>
+    <row r="4" spans="2:36" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="C4" s="170"/>
       <c r="D4" s="108" t="s">
         <v>9</v>
       </c>
@@ -11668,47 +11642,107 @@
       <c r="Q4" s="109" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="5" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="176" t="s">
+      <c r="AB4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AC4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="AD4" s="8"/>
+      <c r="AE4" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG4" s="7" t="s">
+        <v>6</v>
+      </c>
+      <c r="AH4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="AI4" s="8"/>
+      <c r="AJ4" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="168" t="s">
         <v>67</v>
       </c>
       <c r="C5" s="88" t="s">
         <v>21</v>
       </c>
-      <c r="D5" s="111"/>
-      <c r="E5" s="112"/>
-      <c r="F5" s="111"/>
-      <c r="G5" s="112"/>
+      <c r="D5" s="111">
+        <v>1.0337000000000001</v>
+      </c>
+      <c r="E5" s="112">
+        <v>0.1</v>
+      </c>
+      <c r="F5" s="111">
+        <v>0.99980000000000002</v>
+      </c>
+      <c r="G5" s="112">
+        <v>0.09</v>
+      </c>
       <c r="H5" s="113">
-        <f t="shared" ref="H5:H20" si="0">I5/30%</f>
-        <v>0</v>
+        <f>I5/30%</f>
+        <v>1.2200000000000002</v>
       </c>
       <c r="I5" s="114">
-        <f t="shared" ref="I5:I19" si="1">E5+G5+$AI$20+$AK$20</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="156"/>
-      <c r="K5" s="158"/>
-      <c r="L5" s="156"/>
-      <c r="M5" s="158"/>
-      <c r="N5" s="186">
+        <f>E5+G5+$E$20+$G$20</f>
+        <v>0.36600000000000005</v>
+      </c>
+      <c r="J5" s="148">
+        <v>1.0337000000000001</v>
+      </c>
+      <c r="K5" s="150">
+        <v>0</v>
+      </c>
+      <c r="L5" s="148">
+        <v>0.99980000000000002</v>
+      </c>
+      <c r="M5" s="150">
+        <v>0</v>
+      </c>
+      <c r="N5" s="178">
         <v>1.0759000000000001</v>
       </c>
-      <c r="O5" s="183">
+      <c r="O5" s="175">
         <v>7.0000000000000007E-2</v>
       </c>
       <c r="P5" s="113">
-        <f t="shared" ref="P5:P20" si="2">Q5/30%</f>
-        <v>0</v>
+        <f t="shared" ref="P5:P20" si="0">Q5/30%</f>
+        <v>1.5533333333333335</v>
       </c>
       <c r="Q5" s="115">
-        <f t="shared" ref="Q5:Q19" si="3">I5+$AO$5+$AQ$5+$AS$5</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B6" s="177"/>
+        <f>I5+$K$20+$M$20+$O$5</f>
+        <v>0.46600000000000003</v>
+      </c>
+      <c r="AB5" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC5" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD5" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE5" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG5" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH5" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI5" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ5" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="6" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="169"/>
       <c r="C6" s="92" t="s">
         <v>38</v>
       </c>
@@ -11716,31 +11750,55 @@
       <c r="E6" s="117"/>
       <c r="F6" s="116"/>
       <c r="G6" s="118"/>
-      <c r="H6" s="119">
+      <c r="H6" s="113">
+        <f t="shared" ref="H5:H20" si="1">I6/30%</f>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I6" s="114">
+        <f t="shared" ref="I6:I19" si="2">E6+G6+$E$20+$G$20</f>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J6" s="149"/>
+      <c r="K6" s="151"/>
+      <c r="L6" s="149"/>
+      <c r="M6" s="151"/>
+      <c r="N6" s="179"/>
+      <c r="O6" s="176"/>
+      <c r="P6" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I6" s="120">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J6" s="157"/>
-      <c r="K6" s="159"/>
-      <c r="L6" s="157"/>
-      <c r="M6" s="159"/>
-      <c r="N6" s="187"/>
-      <c r="O6" s="184"/>
-      <c r="P6" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q6" s="121">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B7" s="177"/>
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q6" s="115">
+        <f t="shared" ref="Q6:Q19" si="3">I6+$K$20+$M$20+$O$5</f>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB6" s="27">
+        <v>121.1422992</v>
+      </c>
+      <c r="AC6" s="28">
+        <v>0.96</v>
+      </c>
+      <c r="AD6" s="29">
+        <v>0.25</v>
+      </c>
+      <c r="AE6" s="30">
+        <v>1.2500000000000001E-2</v>
+      </c>
+      <c r="AG6" s="27">
+        <v>126.18989500000001</v>
+      </c>
+      <c r="AH6" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI6" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ6" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="169"/>
       <c r="C7" s="92" t="s">
         <v>39</v>
       </c>
@@ -11748,95 +11806,167 @@
       <c r="E7" s="118"/>
       <c r="F7" s="116"/>
       <c r="G7" s="118"/>
-      <c r="H7" s="119">
+      <c r="H7" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I7" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J7" s="149"/>
+      <c r="K7" s="151"/>
+      <c r="L7" s="149"/>
+      <c r="M7" s="151"/>
+      <c r="N7" s="179"/>
+      <c r="O7" s="176"/>
+      <c r="P7" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I7" s="120">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q7" s="115">
+        <f t="shared" si="3"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB7" s="31">
+        <v>121.64705877999999</v>
+      </c>
+      <c r="AC7" s="32">
+        <v>0.96399999999999986</v>
+      </c>
+      <c r="AD7" s="33">
+        <v>0.32464454976303281</v>
+      </c>
+      <c r="AE7" s="34">
+        <v>1.6232227488151642E-2</v>
+      </c>
+      <c r="AG7" s="31">
+        <v>126.61290550000001</v>
+      </c>
+      <c r="AH7" s="32">
+        <v>1.0033521741182208</v>
+      </c>
+      <c r="AI7" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ7" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="8" spans="2:36" ht="15.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="169"/>
+      <c r="C8" s="120" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="121"/>
+      <c r="E8" s="122"/>
+      <c r="F8" s="121"/>
+      <c r="G8" s="123"/>
+      <c r="H8" s="113">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J7" s="157"/>
-      <c r="K7" s="159"/>
-      <c r="L7" s="157"/>
-      <c r="M7" s="159"/>
-      <c r="N7" s="187"/>
-      <c r="O7" s="184"/>
-      <c r="P7" s="119">
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I8" s="114">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q7" s="121">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J8" s="149"/>
+      <c r="K8" s="151"/>
+      <c r="L8" s="149"/>
+      <c r="M8" s="151"/>
+      <c r="N8" s="179"/>
+      <c r="O8" s="176"/>
+      <c r="P8" s="124">
+        <f t="shared" si="0"/>
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q8" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="2:17" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B8" s="177"/>
-      <c r="C8" s="122" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="123"/>
-      <c r="E8" s="124"/>
-      <c r="F8" s="123"/>
-      <c r="G8" s="125"/>
-      <c r="H8" s="126">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I8" s="125">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J8" s="157"/>
-      <c r="K8" s="159"/>
-      <c r="L8" s="157"/>
-      <c r="M8" s="159"/>
-      <c r="N8" s="187"/>
-      <c r="O8" s="184"/>
-      <c r="P8" s="126">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q8" s="127">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B9" s="177"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB8" s="31">
+        <v>122.15181835999999</v>
+      </c>
+      <c r="AC8" s="32">
+        <v>0.96799999999999986</v>
+      </c>
+      <c r="AD8" s="33">
+        <v>0.39928909952606562</v>
+      </c>
+      <c r="AE8" s="34">
+        <v>1.9964454976303281E-2</v>
+      </c>
+      <c r="AG8" s="31">
+        <v>127.03591600000001</v>
+      </c>
+      <c r="AH8" s="32">
+        <v>1.0067043482364417</v>
+      </c>
+      <c r="AI8" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ8" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="9" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="169"/>
       <c r="C9" s="92" t="s">
         <v>41</v>
       </c>
       <c r="D9" s="116"/>
       <c r="E9" s="118"/>
       <c r="F9" s="116"/>
-      <c r="G9" s="128"/>
-      <c r="H9" s="119">
+      <c r="G9" s="125"/>
+      <c r="H9" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I9" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J9" s="149"/>
+      <c r="K9" s="151"/>
+      <c r="L9" s="149"/>
+      <c r="M9" s="151"/>
+      <c r="N9" s="179"/>
+      <c r="O9" s="176"/>
+      <c r="P9" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I9" s="120">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J9" s="157"/>
-      <c r="K9" s="159"/>
-      <c r="L9" s="157"/>
-      <c r="M9" s="159"/>
-      <c r="N9" s="187"/>
-      <c r="O9" s="184"/>
-      <c r="P9" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q9" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q9" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="177"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB9" s="31">
+        <v>122.65657793999999</v>
+      </c>
+      <c r="AC9" s="32">
+        <v>0.97199999999999986</v>
+      </c>
+      <c r="AD9" s="33">
+        <v>0.47393364928910042</v>
+      </c>
+      <c r="AE9" s="34">
+        <v>2.3696682464455023E-2</v>
+      </c>
+      <c r="AG9" s="31">
+        <v>127.45892650000002</v>
+      </c>
+      <c r="AH9" s="32">
+        <v>1.0100565223546625</v>
+      </c>
+      <c r="AI9" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ9" s="34">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="10" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="169"/>
       <c r="C10" s="92" t="s">
         <v>42</v>
       </c>
@@ -11844,364 +11974,2942 @@
       <c r="E10" s="118"/>
       <c r="F10" s="116"/>
       <c r="G10" s="118"/>
-      <c r="H10" s="119">
+      <c r="H10" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I10" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J10" s="149"/>
+      <c r="K10" s="151"/>
+      <c r="L10" s="149"/>
+      <c r="M10" s="151"/>
+      <c r="N10" s="179"/>
+      <c r="O10" s="176"/>
+      <c r="P10" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I10" s="120">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q10" s="115">
+        <f t="shared" si="3"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB10" s="31">
+        <v>123.16133751999999</v>
+      </c>
+      <c r="AC10" s="32">
+        <v>0.97599999999999987</v>
+      </c>
+      <c r="AD10" s="33">
+        <v>0.55035545023696719</v>
+      </c>
+      <c r="AE10" s="34">
+        <v>2.7517772511848362E-2</v>
+      </c>
+      <c r="AG10" s="31">
+        <v>127.88193700000002</v>
+      </c>
+      <c r="AH10" s="32">
+        <v>1.0134086964728832</v>
+      </c>
+      <c r="AI10" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ10" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="2:36" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="170"/>
+      <c r="C11" s="126" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="127"/>
+      <c r="E11" s="128"/>
+      <c r="F11" s="127"/>
+      <c r="G11" s="128"/>
+      <c r="H11" s="113">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J10" s="157"/>
-      <c r="K10" s="159"/>
-      <c r="L10" s="157"/>
-      <c r="M10" s="159"/>
-      <c r="N10" s="187"/>
-      <c r="O10" s="184"/>
-      <c r="P10" s="119">
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I11" s="114">
         <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q10" s="121">
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J11" s="149"/>
+      <c r="K11" s="151"/>
+      <c r="L11" s="149"/>
+      <c r="M11" s="151"/>
+      <c r="N11" s="179"/>
+      <c r="O11" s="176"/>
+      <c r="P11" s="129">
+        <f t="shared" si="0"/>
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q11" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="178"/>
-      <c r="C11" s="129" t="s">
-        <v>43</v>
-      </c>
-      <c r="D11" s="130"/>
-      <c r="E11" s="131"/>
-      <c r="F11" s="130"/>
-      <c r="G11" s="131"/>
-      <c r="H11" s="132">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I11" s="133">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J11" s="157"/>
-      <c r="K11" s="159"/>
-      <c r="L11" s="157"/>
-      <c r="M11" s="159"/>
-      <c r="N11" s="187"/>
-      <c r="O11" s="184"/>
-      <c r="P11" s="132">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q11" s="134">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="176" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB11" s="31">
+        <v>123.66609709999999</v>
+      </c>
+      <c r="AC11" s="32">
+        <v>0.97999999999999987</v>
+      </c>
+      <c r="AD11" s="33">
+        <v>0.625</v>
+      </c>
+      <c r="AE11" s="34">
+        <v>3.125E-2</v>
+      </c>
+      <c r="AG11" s="31">
+        <v>128.30494750000003</v>
+      </c>
+      <c r="AH11" s="32">
+        <v>1.0167608705911042</v>
+      </c>
+      <c r="AI11" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ11" s="34">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="12" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="168" t="s">
         <v>68</v>
       </c>
-      <c r="C12" s="135" t="s">
+      <c r="C12" s="130" t="s">
         <v>48</v>
       </c>
       <c r="D12" s="111"/>
       <c r="E12" s="112"/>
       <c r="F12" s="111"/>
       <c r="G12" s="112"/>
-      <c r="H12" s="136">
+      <c r="H12" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I12" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J12" s="149"/>
+      <c r="K12" s="151"/>
+      <c r="L12" s="149"/>
+      <c r="M12" s="151"/>
+      <c r="N12" s="179"/>
+      <c r="O12" s="176"/>
+      <c r="P12" s="131">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I12" s="114">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J12" s="157"/>
-      <c r="K12" s="159"/>
-      <c r="L12" s="157"/>
-      <c r="M12" s="159"/>
-      <c r="N12" s="187"/>
-      <c r="O12" s="184"/>
-      <c r="P12" s="136">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.92000000000000015</v>
       </c>
       <c r="Q12" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="177"/>
-      <c r="C13" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB12" s="31">
+        <v>124.17085667999999</v>
+      </c>
+      <c r="AC12" s="32">
+        <v>0.98399999999999987</v>
+      </c>
+      <c r="AD12" s="33">
+        <v>0.69964454976303281</v>
+      </c>
+      <c r="AE12" s="34">
+        <v>3.4982227488151642E-2</v>
+      </c>
+      <c r="AG12" s="31">
+        <v>128.72795800000003</v>
+      </c>
+      <c r="AH12" s="32">
+        <v>1.020113044709325</v>
+      </c>
+      <c r="AI12" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ12" s="34">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="13" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="169"/>
+      <c r="C13" s="132" t="s">
         <v>49</v>
       </c>
       <c r="D13" s="116"/>
       <c r="E13" s="117"/>
       <c r="F13" s="116"/>
       <c r="G13" s="117"/>
-      <c r="H13" s="119">
+      <c r="H13" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I13" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J13" s="149"/>
+      <c r="K13" s="151"/>
+      <c r="L13" s="149"/>
+      <c r="M13" s="151"/>
+      <c r="N13" s="179"/>
+      <c r="O13" s="176"/>
+      <c r="P13" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I13" s="117">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J13" s="157"/>
-      <c r="K13" s="159"/>
-      <c r="L13" s="157"/>
-      <c r="M13" s="159"/>
-      <c r="N13" s="187"/>
-      <c r="O13" s="184"/>
-      <c r="P13" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q13" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q13" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="177"/>
-      <c r="C14" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB13" s="31">
+        <v>124.67561625999998</v>
+      </c>
+      <c r="AC13" s="32">
+        <v>0.98799999999999977</v>
+      </c>
+      <c r="AD13" s="33">
+        <v>0.77428909952606562</v>
+      </c>
+      <c r="AE13" s="34">
+        <v>3.8714454976303284E-2</v>
+      </c>
+      <c r="AG13" s="31">
+        <v>129.15096850000003</v>
+      </c>
+      <c r="AH13" s="32">
+        <v>1.0234652188275457</v>
+      </c>
+      <c r="AI13" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ13" s="34">
+        <v>6.9999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="14" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B14" s="169"/>
+      <c r="C14" s="132" t="s">
         <v>50</v>
       </c>
       <c r="D14" s="116"/>
       <c r="E14" s="118"/>
       <c r="F14" s="116"/>
       <c r="G14" s="118"/>
-      <c r="H14" s="119">
+      <c r="H14" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I14" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J14" s="149"/>
+      <c r="K14" s="151"/>
+      <c r="L14" s="149"/>
+      <c r="M14" s="151"/>
+      <c r="N14" s="179"/>
+      <c r="O14" s="176"/>
+      <c r="P14" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I14" s="120">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J14" s="157"/>
-      <c r="K14" s="159"/>
-      <c r="L14" s="157"/>
-      <c r="M14" s="159"/>
-      <c r="N14" s="187"/>
-      <c r="O14" s="184"/>
-      <c r="P14" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q14" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q14" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="177"/>
-      <c r="C15" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB14" s="31">
+        <v>125.18037583999998</v>
+      </c>
+      <c r="AC14" s="32">
+        <v>0.99199999999999977</v>
+      </c>
+      <c r="AD14" s="33">
+        <v>0.85071090047393438</v>
+      </c>
+      <c r="AE14" s="34">
+        <v>4.2535545023696719E-2</v>
+      </c>
+      <c r="AG14" s="31">
+        <v>129.57397900000004</v>
+      </c>
+      <c r="AH14" s="32">
+        <v>1.0268173929457667</v>
+      </c>
+      <c r="AI14" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ14" s="34">
+        <v>8.0000000000000016E-2</v>
+      </c>
+    </row>
+    <row r="15" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="169"/>
+      <c r="C15" s="132" t="s">
         <v>51</v>
       </c>
       <c r="D15" s="116"/>
       <c r="E15" s="117"/>
       <c r="F15" s="116"/>
       <c r="G15" s="118"/>
-      <c r="H15" s="119">
+      <c r="H15" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I15" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J15" s="149"/>
+      <c r="K15" s="151"/>
+      <c r="L15" s="149"/>
+      <c r="M15" s="151"/>
+      <c r="N15" s="179"/>
+      <c r="O15" s="176"/>
+      <c r="P15" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I15" s="120">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J15" s="157"/>
-      <c r="K15" s="159"/>
-      <c r="L15" s="157"/>
-      <c r="M15" s="159"/>
-      <c r="N15" s="187"/>
-      <c r="O15" s="184"/>
-      <c r="P15" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q15" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="177"/>
-      <c r="C16" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB15" s="31">
+        <v>125.68513541999998</v>
+      </c>
+      <c r="AC15" s="32">
+        <v>0.99599999999999977</v>
+      </c>
+      <c r="AD15" s="33">
+        <v>0.92535545023696719</v>
+      </c>
+      <c r="AE15" s="34">
+        <v>4.6267772511848361E-2</v>
+      </c>
+      <c r="AG15" s="31">
+        <v>129.99698950000004</v>
+      </c>
+      <c r="AH15" s="32">
+        <v>1.0301695670639874</v>
+      </c>
+      <c r="AI15" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ15" s="34">
+        <v>9.0000000000000011E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B16" s="169"/>
+      <c r="C16" s="132" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="116"/>
       <c r="E16" s="117"/>
       <c r="F16" s="116"/>
       <c r="G16" s="117"/>
-      <c r="H16" s="119">
+      <c r="H16" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I16" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J16" s="149"/>
+      <c r="K16" s="151"/>
+      <c r="L16" s="149"/>
+      <c r="M16" s="151"/>
+      <c r="N16" s="179"/>
+      <c r="O16" s="176"/>
+      <c r="P16" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I16" s="117">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J16" s="157"/>
-      <c r="K16" s="159"/>
-      <c r="L16" s="157"/>
-      <c r="M16" s="159"/>
-      <c r="N16" s="187"/>
-      <c r="O16" s="184"/>
-      <c r="P16" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q16" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q16" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="177"/>
-      <c r="C17" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB16" s="27">
+        <v>126.18989500000001</v>
+      </c>
+      <c r="AC16" s="40">
+        <v>1</v>
+      </c>
+      <c r="AD16" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE16" s="41">
+        <v>0.05</v>
+      </c>
+      <c r="AG16" s="27">
+        <v>130.41999999999999</v>
+      </c>
+      <c r="AH16" s="42">
+        <v>1.0335217411822077</v>
+      </c>
+      <c r="AI16" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ16" s="41">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="17" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="169"/>
+      <c r="C17" s="132" t="s">
         <v>52</v>
       </c>
       <c r="D17" s="116"/>
       <c r="E17" s="118"/>
       <c r="F17" s="116"/>
       <c r="G17" s="118"/>
-      <c r="H17" s="119">
+      <c r="H17" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I17" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J17" s="149"/>
+      <c r="K17" s="151"/>
+      <c r="L17" s="149"/>
+      <c r="M17" s="151"/>
+      <c r="N17" s="179"/>
+      <c r="O17" s="176"/>
+      <c r="P17" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I17" s="120">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J17" s="157"/>
-      <c r="K17" s="159"/>
-      <c r="L17" s="157"/>
-      <c r="M17" s="159"/>
-      <c r="N17" s="187"/>
-      <c r="O17" s="184"/>
-      <c r="P17" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="121">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q17" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="2:17" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="177"/>
-      <c r="C18" s="137" t="s">
+        <v>0.27600000000000002</v>
+      </c>
+    </row>
+    <row r="18" spans="2:36" ht="14.45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="169"/>
+      <c r="C18" s="132" t="s">
         <v>45</v>
       </c>
       <c r="D18" s="116"/>
       <c r="E18" s="117"/>
       <c r="F18" s="116"/>
       <c r="G18" s="117"/>
-      <c r="H18" s="119">
+      <c r="H18" s="113">
+        <f t="shared" si="1"/>
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I18" s="114">
+        <f t="shared" si="2"/>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J18" s="149"/>
+      <c r="K18" s="151"/>
+      <c r="L18" s="149"/>
+      <c r="M18" s="151"/>
+      <c r="N18" s="179"/>
+      <c r="O18" s="176"/>
+      <c r="P18" s="119">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I18" s="117">
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q18" s="115">
+        <f t="shared" si="3"/>
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB18" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="AC18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="AD18" s="8"/>
+      <c r="AE18" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG18" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="AH18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="AI18" s="8"/>
+      <c r="AJ18" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="2:36" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="170"/>
+      <c r="C19" s="133" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="134"/>
+      <c r="E19" s="135"/>
+      <c r="F19" s="134"/>
+      <c r="G19" s="136"/>
+      <c r="H19" s="113">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J18" s="157"/>
-      <c r="K18" s="159"/>
-      <c r="L18" s="157"/>
-      <c r="M18" s="159"/>
-      <c r="N18" s="187"/>
-      <c r="O18" s="184"/>
-      <c r="P18" s="119">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q18" s="121">
+        <v>0.58666666666666667</v>
+      </c>
+      <c r="I19" s="114">
+        <f>E19+G19+$E$20+$G$20</f>
+        <v>0.17599999999999999</v>
+      </c>
+      <c r="J19" s="149"/>
+      <c r="K19" s="151"/>
+      <c r="L19" s="149"/>
+      <c r="M19" s="151"/>
+      <c r="N19" s="179"/>
+      <c r="O19" s="176"/>
+      <c r="P19" s="137">
+        <f t="shared" si="0"/>
+        <v>0.92000000000000015</v>
+      </c>
+      <c r="Q19" s="115">
         <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="2:17" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="178"/>
-      <c r="C19" s="138" t="s">
-        <v>69</v>
-      </c>
-      <c r="D19" s="139"/>
-      <c r="E19" s="140"/>
-      <c r="F19" s="139"/>
-      <c r="G19" s="141"/>
-      <c r="H19" s="142">
+        <v>0.27600000000000002</v>
+      </c>
+      <c r="AB19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="AC19" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD19" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE19" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG19" s="18" t="s">
+        <v>8</v>
+      </c>
+      <c r="AH19" s="19" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI19" s="20" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ19" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="20" spans="2:36" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B20" s="138"/>
+      <c r="C20" s="139" t="s">
+        <v>47</v>
+      </c>
+      <c r="D20" s="140">
+        <v>1.012977411325948</v>
+      </c>
+      <c r="E20" s="141">
+        <v>9.6000000000000002E-2</v>
+      </c>
+      <c r="F20" s="142">
+        <v>0.99789679989536106</v>
+      </c>
+      <c r="G20" s="143">
+        <v>0.08</v>
+      </c>
+      <c r="H20" s="144">
+        <f>I20/30%</f>
+        <v>0.95</v>
+      </c>
+      <c r="I20" s="145">
+        <v>0.28499999999999998</v>
+      </c>
+      <c r="J20" s="152">
+        <v>1.012977411325948</v>
+      </c>
+      <c r="K20" s="153">
+        <v>0.03</v>
+      </c>
+      <c r="L20" s="152">
+        <v>0.99789679989536106</v>
+      </c>
+      <c r="M20" s="153">
+        <v>0</v>
+      </c>
+      <c r="N20" s="180"/>
+      <c r="O20" s="177"/>
+      <c r="P20" s="144">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="I19" s="143">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="J19" s="157"/>
-      <c r="K19" s="159"/>
-      <c r="L19" s="157"/>
-      <c r="M19" s="159"/>
-      <c r="N19" s="187"/>
-      <c r="O19" s="184"/>
-      <c r="P19" s="144">
-        <f t="shared" si="2"/>
-        <v>0</v>
-      </c>
-      <c r="Q19" s="145">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="2:17" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B20" s="146"/>
-      <c r="C20" s="147" t="s">
-        <v>47</v>
-      </c>
-      <c r="D20" s="148">
-        <v>1.012977411325948</v>
-      </c>
-      <c r="E20" s="149">
-        <v>9.6000000000000002E-2</v>
-      </c>
-      <c r="F20" s="150">
-        <v>0.99789679989536106</v>
-      </c>
-      <c r="G20" s="151">
-        <v>0.08</v>
-      </c>
-      <c r="H20" s="152">
-        <f t="shared" si="0"/>
-        <v>0.95</v>
-      </c>
-      <c r="I20" s="153">
-        <v>0.28499999999999998</v>
-      </c>
-      <c r="J20" s="160">
-        <v>1.012977411325948</v>
-      </c>
-      <c r="K20" s="161">
-        <v>0.03</v>
-      </c>
-      <c r="L20" s="160">
-        <v>0.99789679989536106</v>
-      </c>
-      <c r="M20" s="161">
-        <v>0</v>
-      </c>
-      <c r="N20" s="188"/>
-      <c r="O20" s="185"/>
-      <c r="P20" s="152">
-        <f t="shared" si="2"/>
         <v>1.2833333333333332</v>
       </c>
-      <c r="Q20" s="154">
+      <c r="Q20" s="146">
         <f>I20+K20+M20+O5</f>
         <v>0.38499999999999995</v>
+      </c>
+      <c r="AB20" s="27">
+        <v>121.1422992</v>
+      </c>
+      <c r="AC20" s="28">
+        <v>0.96</v>
+      </c>
+      <c r="AD20" s="29">
+        <v>0.25</v>
+      </c>
+      <c r="AE20" s="30">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AG20" s="27">
+        <v>126.18989500000001</v>
+      </c>
+      <c r="AH20" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI20" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ20" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB21" s="31">
+        <v>121.64705877999999</v>
+      </c>
+      <c r="AC21" s="32">
+        <v>0.96399999999999997</v>
+      </c>
+      <c r="AD21" s="33">
+        <v>0.32464454976303281</v>
+      </c>
+      <c r="AE21" s="34">
+        <v>3.2464454976303285E-2</v>
+      </c>
+      <c r="AG21" s="31">
+        <v>126.61290550000001</v>
+      </c>
+      <c r="AH21" s="32">
+        <v>1.0033521741182208</v>
+      </c>
+      <c r="AI21" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ21" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB22" s="31">
+        <v>122.15181835999999</v>
+      </c>
+      <c r="AC22" s="32">
+        <v>0.96799999999999997</v>
+      </c>
+      <c r="AD22" s="33">
+        <v>0.39928909952606562</v>
+      </c>
+      <c r="AE22" s="34">
+        <v>3.9928909952606562E-2</v>
+      </c>
+      <c r="AG22" s="31">
+        <v>127.03591600000001</v>
+      </c>
+      <c r="AH22" s="32">
+        <v>1.0067043482364417</v>
+      </c>
+      <c r="AI22" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ22" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB23" s="31">
+        <v>122.65657793999999</v>
+      </c>
+      <c r="AC23" s="32">
+        <v>0.97199999999999998</v>
+      </c>
+      <c r="AD23" s="33">
+        <v>0.47393364928910042</v>
+      </c>
+      <c r="AE23" s="34">
+        <v>4.7393364928910046E-2</v>
+      </c>
+      <c r="AG23" s="31">
+        <v>127.45892650000002</v>
+      </c>
+      <c r="AH23" s="32">
+        <v>1.0100565223546625</v>
+      </c>
+      <c r="AI23" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ23" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB24" s="31">
+        <v>123.16133751999999</v>
+      </c>
+      <c r="AC24" s="32">
+        <v>0.97599999999999998</v>
+      </c>
+      <c r="AD24" s="33">
+        <v>0.55035545023696719</v>
+      </c>
+      <c r="AE24" s="34">
+        <v>5.5035545023696723E-2</v>
+      </c>
+      <c r="AG24" s="31">
+        <v>127.88193700000002</v>
+      </c>
+      <c r="AH24" s="32">
+        <v>1.0134086964728832</v>
+      </c>
+      <c r="AI24" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ24" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB25" s="31">
+        <v>123.66609709999999</v>
+      </c>
+      <c r="AC25" s="32">
+        <v>0.98</v>
+      </c>
+      <c r="AD25" s="33">
+        <v>0.625</v>
+      </c>
+      <c r="AE25" s="34">
+        <v>6.25E-2</v>
+      </c>
+      <c r="AG25" s="31">
+        <v>128.30494750000003</v>
+      </c>
+      <c r="AH25" s="32">
+        <v>1.0167608705911042</v>
+      </c>
+      <c r="AI25" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ25" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB26" s="31">
+        <v>124.17085667999999</v>
+      </c>
+      <c r="AC26" s="32">
+        <v>0.9840000000000001</v>
+      </c>
+      <c r="AD26" s="33">
+        <v>0.69964454976303281</v>
+      </c>
+      <c r="AE26" s="34">
+        <v>6.9964454976303284E-2</v>
+      </c>
+      <c r="AG26" s="31">
+        <v>128.72795800000003</v>
+      </c>
+      <c r="AH26" s="32">
+        <v>1.020113044709325</v>
+      </c>
+      <c r="AI26" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ26" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB27" s="31">
+        <v>124.67561625999998</v>
+      </c>
+      <c r="AC27" s="32">
+        <v>0.9880000000000001</v>
+      </c>
+      <c r="AD27" s="33">
+        <v>0.77428909952606562</v>
+      </c>
+      <c r="AE27" s="34">
+        <v>7.7428909952606567E-2</v>
+      </c>
+      <c r="AG27" s="31">
+        <v>129.15096850000003</v>
+      </c>
+      <c r="AH27" s="32">
+        <v>1.0234652188275457</v>
+      </c>
+      <c r="AI27" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ27" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB28" s="31">
+        <v>125.18037583999998</v>
+      </c>
+      <c r="AC28" s="32">
+        <v>0.9920000000000001</v>
+      </c>
+      <c r="AD28" s="33">
+        <v>0.85071090047393438</v>
+      </c>
+      <c r="AE28" s="34">
+        <v>8.5071090047393438E-2</v>
+      </c>
+      <c r="AG28" s="31">
+        <v>129.57397900000004</v>
+      </c>
+      <c r="AH28" s="32">
+        <v>1.0268173929457667</v>
+      </c>
+      <c r="AI28" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ28" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB29" s="31">
+        <v>125.68513541999998</v>
+      </c>
+      <c r="AC29" s="32">
+        <v>0.99600000000000011</v>
+      </c>
+      <c r="AD29" s="33">
+        <v>0.92535545023696719</v>
+      </c>
+      <c r="AE29" s="34">
+        <v>9.2535545023696722E-2</v>
+      </c>
+      <c r="AG29" s="31">
+        <v>129.99698950000004</v>
+      </c>
+      <c r="AH29" s="32">
+        <v>1.0301695670639874</v>
+      </c>
+      <c r="AI29" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ29" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB30" s="27">
+        <v>126.18989500000001</v>
+      </c>
+      <c r="AC30" s="40">
+        <v>1</v>
+      </c>
+      <c r="AD30" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE30" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AG30" s="27">
+        <v>130.41999999999999</v>
+      </c>
+      <c r="AH30" s="42">
+        <v>1.0335217411822077</v>
+      </c>
+      <c r="AI30" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ30" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="2:36" x14ac:dyDescent="0.25">
+      <c r="AB32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="AC32" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="AD32" s="8"/>
+      <c r="AE32" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG32" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="AH32" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="AI32" s="8"/>
+      <c r="AJ32" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="33" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB33" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC33" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD33" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE33" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG33" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH33" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI33" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ33" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="34" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB34" s="27">
+        <v>288.48343914836181</v>
+      </c>
+      <c r="AC34" s="28">
+        <v>0.97299999999999998</v>
+      </c>
+      <c r="AD34" s="29">
+        <v>0</v>
+      </c>
+      <c r="AE34" s="30">
+        <v>0</v>
+      </c>
+      <c r="AG34" s="27">
+        <v>296.48863221825468</v>
+      </c>
+      <c r="AH34" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI34" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ34" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="4:36" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D35" s="82" t="s">
+        <v>55</v>
+      </c>
+      <c r="AB35" s="31">
+        <v>289.28395845535113</v>
+      </c>
+      <c r="AC35" s="32">
+        <v>0.97570000000000012</v>
+      </c>
+      <c r="AD35" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AE35" s="34">
+        <v>5.000000000000001E-3</v>
+      </c>
+      <c r="AG35" s="31">
+        <v>296.65976899642919</v>
+      </c>
+      <c r="AH35" s="32">
+        <v>1.0005772119385965</v>
+      </c>
+      <c r="AI35" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ35" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="36" spans="4:36" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D36" s="84" t="s">
+        <v>27</v>
+      </c>
+      <c r="E36" s="85" t="s">
+        <v>28</v>
+      </c>
+      <c r="F36" s="85" t="s">
+        <v>29</v>
+      </c>
+      <c r="G36" s="85" t="s">
+        <v>30</v>
+      </c>
+      <c r="H36" s="85" t="s">
+        <v>31</v>
+      </c>
+      <c r="I36" s="85" t="s">
+        <v>32</v>
+      </c>
+      <c r="J36" s="85" t="s">
+        <v>33</v>
+      </c>
+      <c r="K36" s="85" t="s">
+        <v>34</v>
+      </c>
+      <c r="L36" s="85" t="s">
+        <v>35</v>
+      </c>
+      <c r="M36" s="86" t="s">
+        <v>36</v>
+      </c>
+      <c r="N36" s="87" t="s">
+        <v>37</v>
+      </c>
+      <c r="O36" s="86" t="s">
+        <v>56</v>
+      </c>
+      <c r="P36" s="105" t="s">
+        <v>57</v>
+      </c>
+      <c r="Q36" s="87" t="s">
+        <v>58</v>
+      </c>
+      <c r="R36" s="86" t="s">
+        <v>59</v>
+      </c>
+      <c r="S36" s="105" t="s">
+        <v>60</v>
+      </c>
+      <c r="T36" s="105" t="s">
+        <v>61</v>
+      </c>
+      <c r="U36" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="V36" s="163"/>
+      <c r="AB36" s="31">
+        <v>290.08447776234038</v>
+      </c>
+      <c r="AC36" s="32">
+        <v>0.97840000000000005</v>
+      </c>
+      <c r="AD36" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AE36" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="AG36" s="31">
+        <v>296.83090577460371</v>
+      </c>
+      <c r="AH36" s="32">
+        <v>1.001154423877193</v>
+      </c>
+      <c r="AI36" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ36" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="37" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D37" s="88" t="s">
+        <v>21</v>
+      </c>
+      <c r="E37" s="89">
+        <v>5531728333.578927</v>
+      </c>
+      <c r="F37" s="89">
+        <v>5722513147.3449001</v>
+      </c>
+      <c r="G37" s="89">
+        <v>243288.48603071459</v>
+      </c>
+      <c r="H37" s="89">
+        <v>243230.2250345443</v>
+      </c>
+      <c r="I37" s="89">
+        <v>3801903908.3698511</v>
+      </c>
+      <c r="J37" s="89">
+        <v>3930190817.9795208</v>
+      </c>
+      <c r="K37" s="89">
+        <v>22737.320716774739</v>
+      </c>
+      <c r="L37" s="89">
+        <v>23527.146540000002</v>
+      </c>
+      <c r="M37" s="100">
+        <f t="shared" ref="M37:M52" si="4">J37/I37</f>
+        <v>1.0337428069466057</v>
+      </c>
+      <c r="N37" s="101">
+        <f t="shared" ref="N37:N52" si="5">H37/G37</f>
+        <v>0.99976052711280827</v>
+      </c>
+      <c r="O37" s="90"/>
+      <c r="Q37" s="91"/>
+      <c r="R37" s="90"/>
+      <c r="T37" s="161"/>
+      <c r="U37" s="164">
+        <v>1.0449999999999999</v>
+      </c>
+      <c r="V37" s="13"/>
+      <c r="AB37" s="31">
+        <v>290.88499706932964</v>
+      </c>
+      <c r="AC37" s="32">
+        <v>0.98109999999999997</v>
+      </c>
+      <c r="AD37" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AE37" s="34">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="AG37" s="31">
+        <v>297.00204255277822</v>
+      </c>
+      <c r="AH37" s="32">
+        <v>1.0017316358157895</v>
+      </c>
+      <c r="AI37" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ37" s="34">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="38" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D38" s="92" t="s">
+        <v>38</v>
+      </c>
+      <c r="E38" s="89">
+        <v>25887293235.70483</v>
+      </c>
+      <c r="F38" s="89">
+        <v>25772150539.867569</v>
+      </c>
+      <c r="G38" s="89">
+        <v>302140.62880146049</v>
+      </c>
+      <c r="H38" s="89">
+        <v>303858.0123632708</v>
+      </c>
+      <c r="I38" s="89">
+        <v>16786195553.83762</v>
+      </c>
+      <c r="J38" s="89">
+        <v>16598168561.750509</v>
+      </c>
+      <c r="K38" s="89">
+        <v>85679.616602359092</v>
+      </c>
+      <c r="L38" s="89">
+        <v>84816.425735900091</v>
+      </c>
+      <c r="M38" s="100">
+        <f t="shared" si="4"/>
+        <v>0.98879871311613998</v>
+      </c>
+      <c r="N38" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0056840537091052</v>
+      </c>
+      <c r="O38" s="90"/>
+      <c r="Q38" s="91"/>
+      <c r="R38" s="90"/>
+      <c r="T38" s="161"/>
+      <c r="U38" s="23"/>
+      <c r="V38" s="13"/>
+      <c r="AB38" s="31">
+        <v>291.6855163763189</v>
+      </c>
+      <c r="AC38" s="32">
+        <v>0.98379999999999979</v>
+      </c>
+      <c r="AD38" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AE38" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+      <c r="AG38" s="31">
+        <v>297.17317933095273</v>
+      </c>
+      <c r="AH38" s="32">
+        <v>1.0023088477543858</v>
+      </c>
+      <c r="AI38" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ38" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+    </row>
+    <row r="39" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D39" s="92" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39" s="89">
+        <v>39033133468.757896</v>
+      </c>
+      <c r="F39" s="89">
+        <v>41008799933.206749</v>
+      </c>
+      <c r="G39" s="89">
+        <v>321633.07344217342</v>
+      </c>
+      <c r="H39" s="89">
+        <v>322273.92237753549</v>
+      </c>
+      <c r="I39" s="89">
+        <v>25237711707.1982</v>
+      </c>
+      <c r="J39" s="89">
+        <v>26145328798.881561</v>
+      </c>
+      <c r="K39" s="89">
+        <v>121359.2030540221</v>
+      </c>
+      <c r="L39" s="89">
+        <v>127248.2726206001</v>
+      </c>
+      <c r="M39" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0359627331595398</v>
+      </c>
+      <c r="N39" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0019924845679071</v>
+      </c>
+      <c r="O39" s="90"/>
+      <c r="Q39" s="91"/>
+      <c r="R39" s="90"/>
+      <c r="T39" s="161"/>
+      <c r="U39" s="23"/>
+      <c r="V39" s="13"/>
+      <c r="AB39" s="31">
+        <v>292.48603568330816</v>
+      </c>
+      <c r="AC39" s="32">
+        <v>0.98649999999999971</v>
+      </c>
+      <c r="AD39" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AE39" s="34">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AG39" s="31">
+        <v>297.34431610912725</v>
+      </c>
+      <c r="AH39" s="32">
+        <v>1.0028860596929823</v>
+      </c>
+      <c r="AI39" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ39" s="34">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="40" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D40" s="92" t="s">
+        <v>40</v>
+      </c>
+      <c r="E40" s="89">
+        <v>39064986435.173508</v>
+      </c>
+      <c r="F40" s="89">
+        <v>38387249190.441788</v>
+      </c>
+      <c r="G40" s="89">
+        <v>281289.45081007812</v>
+      </c>
+      <c r="H40" s="89">
+        <v>279681.81026483118</v>
+      </c>
+      <c r="I40" s="89">
+        <v>25366348050.97403</v>
+      </c>
+      <c r="J40" s="89">
+        <v>25493634341.00856</v>
+      </c>
+      <c r="K40" s="89">
+        <v>138878.24915819379</v>
+      </c>
+      <c r="L40" s="89">
+        <v>137253.29206820001</v>
+      </c>
+      <c r="M40" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0050179194016713</v>
+      </c>
+      <c r="N40" s="101">
+        <f t="shared" si="5"/>
+        <v>0.99428474640404341</v>
+      </c>
+      <c r="O40" s="90"/>
+      <c r="Q40" s="91"/>
+      <c r="R40" s="90"/>
+      <c r="T40" s="161"/>
+      <c r="U40" s="23"/>
+      <c r="V40" s="13"/>
+      <c r="AB40" s="31">
+        <v>293.28655499029742</v>
+      </c>
+      <c r="AC40" s="32">
+        <v>0.98919999999999964</v>
+      </c>
+      <c r="AD40" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AE40" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="AG40" s="31">
+        <v>297.51545288730176</v>
+      </c>
+      <c r="AH40" s="32">
+        <v>1.0034632716315788</v>
+      </c>
+      <c r="AI40" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ40" s="34">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="41" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D41" s="92" t="s">
+        <v>41</v>
+      </c>
+      <c r="E41" s="89">
+        <v>31363293942.790661</v>
+      </c>
+      <c r="F41" s="89">
+        <v>32231379532.868431</v>
+      </c>
+      <c r="G41" s="89">
+        <v>300298.32964414719</v>
+      </c>
+      <c r="H41" s="89">
+        <v>299612.13457182533</v>
+      </c>
+      <c r="I41" s="89">
+        <v>20223911926.343941</v>
+      </c>
+      <c r="J41" s="89">
+        <v>20947521799.438931</v>
+      </c>
+      <c r="K41" s="89">
+        <v>104440.4541975178</v>
+      </c>
+      <c r="L41" s="89">
+        <v>107577.0164614</v>
+      </c>
+      <c r="M41" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0357799161571903</v>
+      </c>
+      <c r="N41" s="101">
+        <f t="shared" si="5"/>
+        <v>0.99771495541405442</v>
+      </c>
+      <c r="O41" s="90"/>
+      <c r="Q41" s="91"/>
+      <c r="R41" s="90"/>
+      <c r="T41" s="161"/>
+      <c r="U41" s="23"/>
+      <c r="V41" s="13"/>
+      <c r="AB41" s="31">
+        <v>294.08707429728668</v>
+      </c>
+      <c r="AC41" s="32">
+        <v>0.99189999999999956</v>
+      </c>
+      <c r="AD41" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AE41" s="34">
+        <v>3.4999999999999996E-2</v>
+      </c>
+      <c r="AG41" s="31">
+        <v>297.68658966547628</v>
+      </c>
+      <c r="AH41" s="32">
+        <v>1.0040404835701753</v>
+      </c>
+      <c r="AI41" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ41" s="34">
+        <v>6.9999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="42" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D42" s="92" t="s">
+        <v>42</v>
+      </c>
+      <c r="E42" s="89">
+        <v>15824782777.47311</v>
+      </c>
+      <c r="F42" s="89">
+        <v>16024483305.16786</v>
+      </c>
+      <c r="G42" s="89">
+        <v>297056.50566868781</v>
+      </c>
+      <c r="H42" s="89">
+        <v>299534.58118034771</v>
+      </c>
+      <c r="I42" s="89">
+        <v>10549369205.51005</v>
+      </c>
+      <c r="J42" s="89">
+        <v>10734741236.254009</v>
+      </c>
+      <c r="K42" s="89">
+        <v>53271.961648679593</v>
+      </c>
+      <c r="L42" s="89">
+        <v>53497.940845500023</v>
+      </c>
+      <c r="M42" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0175718592394261</v>
+      </c>
+      <c r="N42" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0083421014667955</v>
+      </c>
+      <c r="O42" s="90"/>
+      <c r="Q42" s="91"/>
+      <c r="R42" s="90"/>
+      <c r="T42" s="161"/>
+      <c r="U42" s="23"/>
+      <c r="V42" s="13"/>
+      <c r="AB42" s="31">
+        <v>294.88759360427593</v>
+      </c>
+      <c r="AC42" s="32">
+        <v>0.99459999999999948</v>
+      </c>
+      <c r="AD42" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AE42" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="AG42" s="31">
+        <v>297.85772644365079</v>
+      </c>
+      <c r="AH42" s="32">
+        <v>1.0046176955087718</v>
+      </c>
+      <c r="AI42" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ42" s="34">
+        <v>8.0000000000000016E-2</v>
+      </c>
+    </row>
+    <row r="43" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D43" s="92" t="s">
+        <v>43</v>
+      </c>
+      <c r="E43" s="89">
+        <v>9610027969.7755451</v>
+      </c>
+      <c r="F43" s="89">
+        <v>10345034022.67058</v>
+      </c>
+      <c r="G43" s="89">
+        <v>269605.32289907231</v>
+      </c>
+      <c r="H43" s="89">
+        <v>270583.76679249608</v>
+      </c>
+      <c r="I43" s="89">
+        <v>7109195907.7456074</v>
+      </c>
+      <c r="J43" s="89">
+        <v>7708744707.4835024</v>
+      </c>
+      <c r="K43" s="89">
+        <v>35644.800579004492</v>
+      </c>
+      <c r="L43" s="89">
+        <v>38232.278844000008</v>
+      </c>
+      <c r="M43" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0843342633285256</v>
+      </c>
+      <c r="N43" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0036291712748937</v>
+      </c>
+      <c r="O43" s="90"/>
+      <c r="Q43" s="91"/>
+      <c r="R43" s="90"/>
+      <c r="T43" s="161"/>
+      <c r="U43" s="23"/>
+      <c r="V43" s="13"/>
+      <c r="AB43" s="31">
+        <v>295.68811291126519</v>
+      </c>
+      <c r="AC43" s="32">
+        <v>0.9972999999999993</v>
+      </c>
+      <c r="AD43" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AE43" s="34">
+        <v>4.5000000000000005E-2</v>
+      </c>
+      <c r="AG43" s="31">
+        <v>298.0288632218253</v>
+      </c>
+      <c r="AH43" s="32">
+        <v>1.0051949074473683</v>
+      </c>
+      <c r="AI43" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ43" s="34">
+        <v>9.0000000000000011E-2</v>
+      </c>
+    </row>
+    <row r="44" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D44" s="92" t="s">
+        <v>44</v>
+      </c>
+      <c r="E44" s="89">
+        <v>9682802485.2179852</v>
+      </c>
+      <c r="F44" s="89">
+        <v>7998082662.0638533</v>
+      </c>
+      <c r="G44" s="89">
+        <v>281970.03450858378</v>
+      </c>
+      <c r="H44" s="89">
+        <v>279175.33649261057</v>
+      </c>
+      <c r="I44" s="89">
+        <v>6952879491.9023466</v>
+      </c>
+      <c r="J44" s="89">
+        <v>5756977484.97264</v>
+      </c>
+      <c r="K44" s="89">
+        <v>34339.827996592372</v>
+      </c>
+      <c r="L44" s="89">
+        <v>28648.958617</v>
+      </c>
+      <c r="M44" s="100">
+        <f t="shared" si="4"/>
+        <v>0.8279990314340252</v>
+      </c>
+      <c r="N44" s="101">
+        <f t="shared" si="5"/>
+        <v>0.99008867016367963</v>
+      </c>
+      <c r="O44" s="90"/>
+      <c r="Q44" s="91"/>
+      <c r="R44" s="90"/>
+      <c r="T44" s="161"/>
+      <c r="U44" s="23"/>
+      <c r="V44" s="13"/>
+      <c r="AB44" s="78">
+        <v>296.48863221825468</v>
+      </c>
+      <c r="AC44" s="40">
+        <v>1</v>
+      </c>
+      <c r="AD44" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE44" s="41">
+        <v>0.05</v>
+      </c>
+      <c r="AG44" s="78">
+        <v>298.2</v>
+      </c>
+      <c r="AH44" s="42">
+        <v>1.0057721193859652</v>
+      </c>
+      <c r="AI44" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ44" s="41">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="45" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D45" s="92" t="s">
+        <v>45</v>
+      </c>
+      <c r="E45" s="89">
+        <v>13209596112.34861</v>
+      </c>
+      <c r="F45" s="89">
+        <v>13154398249.22537</v>
+      </c>
+      <c r="G45" s="89">
+        <v>318918.84352995933</v>
+      </c>
+      <c r="H45" s="89">
+        <v>312380.19214124721</v>
+      </c>
+      <c r="I45" s="89">
+        <v>9053750849.0866508</v>
+      </c>
+      <c r="J45" s="89">
+        <v>9007473756.4775219</v>
+      </c>
+      <c r="K45" s="89">
+        <v>41419.929804516883</v>
+      </c>
+      <c r="L45" s="89">
+        <v>42110.218830000013</v>
+      </c>
+      <c r="M45" s="100">
+        <f t="shared" si="4"/>
+        <v>0.99488862755552887</v>
+      </c>
+      <c r="N45" s="101">
+        <f t="shared" si="5"/>
+        <v>0.97949744418881335</v>
+      </c>
+      <c r="O45" s="90"/>
+      <c r="Q45" s="91"/>
+      <c r="R45" s="90"/>
+      <c r="T45" s="161"/>
+      <c r="U45" s="23"/>
+      <c r="V45" s="13"/>
+    </row>
+    <row r="46" spans="4:36" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D46" s="93" t="s">
+        <v>46</v>
+      </c>
+      <c r="E46" s="89">
+        <v>1632345969.9116709</v>
+      </c>
+      <c r="F46" s="89">
+        <v>2004357617.054924</v>
+      </c>
+      <c r="G46" s="89">
+        <v>276866.89024291473</v>
+      </c>
+      <c r="H46" s="89">
+        <v>243701.37482005611</v>
+      </c>
+      <c r="I46" s="89">
+        <v>1108628399.0317249</v>
+      </c>
+      <c r="J46" s="89">
+        <v>1504731668.346525</v>
+      </c>
+      <c r="K46" s="89">
+        <v>5895.778901115621</v>
+      </c>
+      <c r="L46" s="89">
+        <v>8224.6463260000019</v>
+      </c>
+      <c r="M46" s="100">
+        <f t="shared" si="4"/>
+        <v>1.3572912886416733</v>
+      </c>
+      <c r="N46" s="101">
+        <f t="shared" si="5"/>
+        <v>0.88021133406829477</v>
+      </c>
+      <c r="O46" s="90"/>
+      <c r="Q46" s="91"/>
+      <c r="R46" s="90"/>
+      <c r="T46" s="161"/>
+      <c r="U46" s="23"/>
+      <c r="V46" s="13"/>
+      <c r="AB46" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="AC46" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="AD46" s="8"/>
+      <c r="AE46" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG46" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="AH46" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="AI46" s="8"/>
+      <c r="AJ46" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="47" spans="4:36" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D47" s="94" t="s">
+        <v>47</v>
+      </c>
+      <c r="E47" s="95">
+        <v>190839990730.7327</v>
+      </c>
+      <c r="F47" s="95">
+        <v>192648448199.9118</v>
+      </c>
+      <c r="G47" s="95">
+        <v>296488.6322182545</v>
+      </c>
+      <c r="H47" s="95">
+        <v>295865.05729594879</v>
+      </c>
+      <c r="I47" s="95">
+        <v>126189895000</v>
+      </c>
+      <c r="J47" s="95">
+        <v>127827513172.5932</v>
+      </c>
+      <c r="K47" s="95">
+        <v>643667.14265877649</v>
+      </c>
+      <c r="L47" s="95">
+        <v>651136.19688859989</v>
+      </c>
+      <c r="M47" s="96">
+        <f t="shared" si="4"/>
+        <v>1.012977411325948</v>
+      </c>
+      <c r="N47" s="97">
+        <f t="shared" si="5"/>
+        <v>0.99789679989536095</v>
+      </c>
+      <c r="O47" s="95">
+        <v>37141</v>
+      </c>
+      <c r="P47" s="106">
+        <v>39961</v>
+      </c>
+      <c r="Q47" s="97">
+        <f>P47/O47</f>
+        <v>1.0759268732667402</v>
+      </c>
+      <c r="R47" s="95">
+        <v>40439</v>
+      </c>
+      <c r="S47" s="106">
+        <v>40933</v>
+      </c>
+      <c r="T47" s="162">
+        <f>S47/R47</f>
+        <v>1.0122159301664235</v>
+      </c>
+      <c r="U47" s="164">
+        <v>1.034</v>
+      </c>
+      <c r="V47" s="1"/>
+      <c r="AB47" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC47" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD47" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE47" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG47" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH47" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI47" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ47" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="48" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D48" s="88" t="s">
+        <v>48</v>
+      </c>
+      <c r="E48" s="89">
+        <v>51757772702.996872</v>
+      </c>
+      <c r="F48" s="89">
+        <v>52905286701.472458</v>
+      </c>
+      <c r="G48" s="89">
+        <v>329493.68063882372</v>
+      </c>
+      <c r="H48" s="89">
+        <v>331338.21313586831</v>
+      </c>
+      <c r="I48" s="89">
+        <v>33056124115.70142</v>
+      </c>
+      <c r="J48" s="89">
+        <v>33788296905.055</v>
+      </c>
+      <c r="K48" s="89">
+        <v>157082.7476953388</v>
+      </c>
+      <c r="L48" s="89">
+        <v>159671.5519189999</v>
+      </c>
+      <c r="M48" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0221493840835927</v>
+      </c>
+      <c r="N48" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0055980815579479</v>
+      </c>
+      <c r="O48" s="90"/>
+      <c r="Q48" s="91"/>
+      <c r="R48" s="90"/>
+      <c r="T48" s="161"/>
+      <c r="U48" s="23"/>
+      <c r="V48" s="13"/>
+      <c r="AB48" s="27">
+        <v>288.48343914836181</v>
+      </c>
+      <c r="AC48" s="28">
+        <v>0.97299999999999998</v>
+      </c>
+      <c r="AD48" s="29">
+        <v>0</v>
+      </c>
+      <c r="AE48" s="30">
+        <v>0</v>
+      </c>
+      <c r="AG48" s="27">
+        <v>296.48863221825468</v>
+      </c>
+      <c r="AH48" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI48" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ48" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D49" s="92" t="s">
+        <v>49</v>
+      </c>
+      <c r="E49" s="89">
+        <v>51175940436.793243</v>
+      </c>
+      <c r="F49" s="89">
+        <v>49985677539.201103</v>
+      </c>
+      <c r="G49" s="89">
+        <v>323820.57736147032</v>
+      </c>
+      <c r="H49" s="89">
+        <v>322569.15207353811</v>
+      </c>
+      <c r="I49" s="89">
+        <v>29721126093.8307</v>
+      </c>
+      <c r="J49" s="89">
+        <v>28993285879.456459</v>
+      </c>
+      <c r="K49" s="89">
+        <v>158037.95068794291</v>
+      </c>
+      <c r="L49" s="89">
+        <v>154961.12141499991</v>
+      </c>
+      <c r="M49" s="100">
+        <f t="shared" si="4"/>
+        <v>0.97551101488966396</v>
+      </c>
+      <c r="N49" s="101">
+        <f t="shared" si="5"/>
+        <v>0.99613543617848821</v>
+      </c>
+      <c r="O49" s="90"/>
+      <c r="Q49" s="91"/>
+      <c r="R49" s="90"/>
+      <c r="T49" s="161"/>
+      <c r="U49" s="23"/>
+      <c r="V49" s="13"/>
+      <c r="AB49" s="31">
+        <v>289.28395845535113</v>
+      </c>
+      <c r="AC49" s="32">
+        <v>0.97570000000000012</v>
+      </c>
+      <c r="AD49" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AE49" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="AG49" s="31">
+        <v>296.65976899642919</v>
+      </c>
+      <c r="AH49" s="32">
+        <v>1.0005772119385965</v>
+      </c>
+      <c r="AI49" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ49" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D50" s="92" t="s">
+        <v>50</v>
+      </c>
+      <c r="E50" s="89">
+        <v>6603039091.5535774</v>
+      </c>
+      <c r="F50" s="89">
+        <v>7124194665.742135</v>
+      </c>
+      <c r="G50" s="89">
+        <v>304212.50262109691</v>
+      </c>
+      <c r="H50" s="89">
+        <v>307586.90861289093</v>
+      </c>
+      <c r="I50" s="89">
+        <v>4778156883.8152866</v>
+      </c>
+      <c r="J50" s="89">
+        <v>5160048414.3100338</v>
+      </c>
+      <c r="K50" s="89">
+        <v>21705.350814518632</v>
+      </c>
+      <c r="L50" s="89">
+        <v>23161.56658900002</v>
+      </c>
+      <c r="M50" s="100">
+        <f t="shared" si="4"/>
+        <v>1.0799244436255957</v>
+      </c>
+      <c r="N50" s="101">
+        <f t="shared" si="5"/>
+        <v>1.011092265974344</v>
+      </c>
+      <c r="O50" s="90"/>
+      <c r="Q50" s="91"/>
+      <c r="R50" s="90"/>
+      <c r="T50" s="161"/>
+      <c r="U50" s="23"/>
+      <c r="V50" s="13"/>
+      <c r="AB50" s="31">
+        <v>290.08447776234038</v>
+      </c>
+      <c r="AC50" s="32">
+        <v>0.97840000000000005</v>
+      </c>
+      <c r="AD50" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AE50" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+      <c r="AG50" s="31">
+        <v>296.83090577460371</v>
+      </c>
+      <c r="AH50" s="32">
+        <v>1.001154423877193</v>
+      </c>
+      <c r="AI50" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ50" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="4:36" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="D51" s="92" t="s">
+        <v>51</v>
+      </c>
+      <c r="E51" s="89">
+        <v>10538999654.257351</v>
+      </c>
+      <c r="F51" s="89">
+        <v>10398141898.22641</v>
+      </c>
+      <c r="G51" s="89">
+        <v>290538.88454409642</v>
+      </c>
+      <c r="H51" s="89">
+        <v>292173.65985430247</v>
+      </c>
+      <c r="I51" s="89">
+        <v>7666912091.2996349</v>
+      </c>
+      <c r="J51" s="89">
+        <v>7591578187.2053709</v>
+      </c>
+      <c r="K51" s="89">
+        <v>36273.973002941719</v>
+      </c>
+      <c r="L51" s="89">
+        <v>35588.909360999991</v>
+      </c>
+      <c r="M51" s="100">
+        <f t="shared" si="4"/>
+        <v>0.99017415314051238</v>
+      </c>
+      <c r="N51" s="101">
+        <f t="shared" si="5"/>
+        <v>1.0056267005801005</v>
+      </c>
+      <c r="O51" s="90"/>
+      <c r="Q51" s="91"/>
+      <c r="R51" s="90"/>
+      <c r="T51" s="161"/>
+      <c r="U51" s="23"/>
+      <c r="V51" s="13"/>
+      <c r="AB51" s="31">
+        <v>290.88499706932964</v>
+      </c>
+      <c r="AC51" s="32">
+        <v>0.98109999999999997</v>
+      </c>
+      <c r="AD51" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AE51" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="AG51" s="31">
+        <v>297.00204255277822</v>
+      </c>
+      <c r="AH51" s="32">
+        <v>1.0017316358157895</v>
+      </c>
+      <c r="AI51" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ51" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="4:36" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="D52" s="93" t="s">
+        <v>52</v>
+      </c>
+      <c r="E52" s="89">
+        <f>SUM(E48:E51)</f>
+        <v>120075751885.60104</v>
+      </c>
+      <c r="F52" s="89">
+        <f>SUM(F48:F51)</f>
+        <v>120413300804.64211</v>
+      </c>
+      <c r="G52" s="102">
+        <f>E52/K52</f>
+        <v>321832.60450463259</v>
+      </c>
+      <c r="H52" s="102">
+        <f>F52/L52</f>
+        <v>322492.59516811848</v>
+      </c>
+      <c r="I52" s="89">
+        <f>SUM(I48:I51)</f>
+        <v>75222319184.647034</v>
+      </c>
+      <c r="J52" s="89">
+        <f>SUM(J48:J51)</f>
+        <v>75533209386.026871</v>
+      </c>
+      <c r="K52" s="89">
+        <f>SUM(K48:K51)</f>
+        <v>373100.02220074204</v>
+      </c>
+      <c r="L52" s="89">
+        <f>SUM(L48:L51)</f>
+        <v>373383.14928399981</v>
+      </c>
+      <c r="M52" s="103">
+        <f t="shared" si="4"/>
+        <v>1.0041329515594528</v>
+      </c>
+      <c r="N52" s="104">
+        <f t="shared" si="5"/>
+        <v>1.0020507265399718</v>
+      </c>
+      <c r="O52" s="98"/>
+      <c r="P52" s="107"/>
+      <c r="Q52" s="99"/>
+      <c r="R52" s="98"/>
+      <c r="S52" s="107"/>
+      <c r="T52" s="107"/>
+      <c r="U52" s="23"/>
+      <c r="V52" s="13"/>
+      <c r="AB52" s="31">
+        <v>291.6855163763189</v>
+      </c>
+      <c r="AC52" s="32">
+        <v>0.98379999999999979</v>
+      </c>
+      <c r="AD52" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AE52" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="AG52" s="31">
+        <v>297.17317933095273</v>
+      </c>
+      <c r="AH52" s="32">
+        <v>1.0023088477543858</v>
+      </c>
+      <c r="AI52" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ52" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB53" s="31">
+        <v>292.48603568330816</v>
+      </c>
+      <c r="AC53" s="32">
+        <v>0.98649999999999971</v>
+      </c>
+      <c r="AD53" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AE53" s="34">
+        <v>0.05</v>
+      </c>
+      <c r="AG53" s="31">
+        <v>297.34431610912725</v>
+      </c>
+      <c r="AH53" s="32">
+        <v>1.0028860596929823</v>
+      </c>
+      <c r="AI53" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ53" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB54" s="31">
+        <v>293.28655499029742</v>
+      </c>
+      <c r="AC54" s="32">
+        <v>0.98919999999999964</v>
+      </c>
+      <c r="AD54" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AE54" s="34">
+        <v>0.06</v>
+      </c>
+      <c r="AG54" s="31">
+        <v>297.51545288730176</v>
+      </c>
+      <c r="AH54" s="32">
+        <v>1.0034632716315788</v>
+      </c>
+      <c r="AI54" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ54" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB55" s="31">
+        <v>294.08707429728668</v>
+      </c>
+      <c r="AC55" s="32">
+        <v>0.99189999999999956</v>
+      </c>
+      <c r="AD55" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AE55" s="34">
+        <v>6.9999999999999993E-2</v>
+      </c>
+      <c r="AG55" s="31">
+        <v>297.68658966547628</v>
+      </c>
+      <c r="AH55" s="32">
+        <v>1.0040404835701753</v>
+      </c>
+      <c r="AI55" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ55" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB56" s="31">
+        <v>294.88759360427593</v>
+      </c>
+      <c r="AC56" s="32">
+        <v>0.99459999999999948</v>
+      </c>
+      <c r="AD56" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AE56" s="34">
+        <v>8.0000000000000016E-2</v>
+      </c>
+      <c r="AG56" s="31">
+        <v>297.85772644365079</v>
+      </c>
+      <c r="AH56" s="32">
+        <v>1.0046176955087718</v>
+      </c>
+      <c r="AI56" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ56" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB57" s="31">
+        <v>295.68811291126519</v>
+      </c>
+      <c r="AC57" s="32">
+        <v>0.9972999999999993</v>
+      </c>
+      <c r="AD57" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AE57" s="34">
+        <v>9.0000000000000011E-2</v>
+      </c>
+      <c r="AG57" s="31">
+        <v>298.0288632218253</v>
+      </c>
+      <c r="AH57" s="32">
+        <v>1.0051949074473683</v>
+      </c>
+      <c r="AI57" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ57" s="34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB58" s="78">
+        <v>296.48863221825468</v>
+      </c>
+      <c r="AC58" s="40">
+        <v>1</v>
+      </c>
+      <c r="AD58" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE58" s="41">
+        <v>0.1</v>
+      </c>
+      <c r="AG58" s="78">
+        <v>298.2</v>
+      </c>
+      <c r="AH58" s="42">
+        <v>1.0057721193859652</v>
+      </c>
+      <c r="AI58" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ58" s="41">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB60" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AC60" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="AD60" s="8"/>
+      <c r="AE60" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG60" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="AH60" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="AI60" s="8"/>
+      <c r="AJ60" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="61" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB61" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC61" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD61" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE61" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG61" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH61" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI61" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ61" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="62" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB62" s="27">
+        <v>36.138192999999994</v>
+      </c>
+      <c r="AC62" s="79">
+        <v>1</v>
+      </c>
+      <c r="AD62" s="29">
+        <v>0</v>
+      </c>
+      <c r="AE62" s="30">
+        <v>0</v>
+      </c>
+      <c r="AG62" s="27">
+        <v>37.140999999999998</v>
+      </c>
+      <c r="AH62" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI62" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ62" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB63" s="31">
+        <v>36.238473699999993</v>
+      </c>
+      <c r="AC63" s="79">
+        <v>1.0027749229188079</v>
+      </c>
+      <c r="AD63" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AE63" s="34">
+        <v>5.000000000000001E-3</v>
+      </c>
+      <c r="AG63" s="31">
+        <v>37.5124</v>
+      </c>
+      <c r="AH63" s="32">
+        <v>1.0099997307557687</v>
+      </c>
+      <c r="AI63" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ63" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="4:36" x14ac:dyDescent="0.25">
+      <c r="AB64" s="31">
+        <v>36.338754399999992</v>
+      </c>
+      <c r="AC64" s="79">
+        <v>1.0055498458376155</v>
+      </c>
+      <c r="AD64" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AE64" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="AG64" s="31">
+        <v>37.883800000000001</v>
+      </c>
+      <c r="AH64" s="32">
+        <v>1.0199994615115371</v>
+      </c>
+      <c r="AI64" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ64" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="65" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB65" s="31">
+        <v>36.439035099999991</v>
+      </c>
+      <c r="AC65" s="79">
+        <v>1.0083247687564234</v>
+      </c>
+      <c r="AD65" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AE65" s="34">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="AG65" s="31">
+        <v>38.255200000000002</v>
+      </c>
+      <c r="AH65" s="32">
+        <v>1.0299991922673057</v>
+      </c>
+      <c r="AI65" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ65" s="34">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="66" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB66" s="31">
+        <v>36.53931579999999</v>
+      </c>
+      <c r="AC66" s="79">
+        <v>1.0110996916752311</v>
+      </c>
+      <c r="AD66" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AE66" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+      <c r="AG66" s="31">
+        <v>38.626600000000003</v>
+      </c>
+      <c r="AH66" s="32">
+        <v>1.0399989230230744</v>
+      </c>
+      <c r="AI66" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ66" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+    </row>
+    <row r="67" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB67" s="31">
+        <v>36.639596499999989</v>
+      </c>
+      <c r="AC67" s="79">
+        <v>1.0138746145940389</v>
+      </c>
+      <c r="AD67" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AE67" s="34">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AG67" s="31">
+        <v>38.998000000000005</v>
+      </c>
+      <c r="AH67" s="32">
+        <v>1.049998653778843</v>
+      </c>
+      <c r="AI67" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ67" s="34">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="68" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB68" s="31">
+        <v>36.739877199999988</v>
+      </c>
+      <c r="AC68" s="79">
+        <v>1.0166495375128468</v>
+      </c>
+      <c r="AD68" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AE68" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="AG68" s="31">
+        <v>39.369400000000006</v>
+      </c>
+      <c r="AH68" s="32">
+        <v>1.0599983845346115</v>
+      </c>
+      <c r="AI68" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ68" s="34">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="69" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB69" s="31">
+        <v>36.840157899999987</v>
+      </c>
+      <c r="AC69" s="79">
+        <v>1.0194244604316545</v>
+      </c>
+      <c r="AD69" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AE69" s="34">
+        <v>3.4999999999999996E-2</v>
+      </c>
+      <c r="AG69" s="31">
+        <v>39.740800000000007</v>
+      </c>
+      <c r="AH69" s="32">
+        <v>1.0699981152903801</v>
+      </c>
+      <c r="AI69" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ69" s="34">
+        <v>6.9999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="70" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB70" s="31">
+        <v>36.940438599999986</v>
+      </c>
+      <c r="AC70" s="79">
+        <v>1.0221993833504623</v>
+      </c>
+      <c r="AD70" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AE70" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="AG70" s="31">
+        <v>40.112200000000009</v>
+      </c>
+      <c r="AH70" s="32">
+        <v>1.0799978460461488</v>
+      </c>
+      <c r="AI70" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ70" s="34">
+        <v>8.0000000000000016E-2</v>
+      </c>
+    </row>
+    <row r="71" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB71" s="31">
+        <v>37.040719299999985</v>
+      </c>
+      <c r="AC71" s="79">
+        <v>1.02497430626927</v>
+      </c>
+      <c r="AD71" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AE71" s="34">
+        <v>4.5000000000000005E-2</v>
+      </c>
+      <c r="AG71" s="31">
+        <v>40.48360000000001</v>
+      </c>
+      <c r="AH71" s="32">
+        <v>1.0899975768019174</v>
+      </c>
+      <c r="AI71" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ71" s="34">
+        <v>9.0000000000000011E-2</v>
+      </c>
+    </row>
+    <row r="72" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB72" s="78">
+        <v>37.140999999999998</v>
+      </c>
+      <c r="AC72" s="79">
+        <v>1.0277492291880783</v>
+      </c>
+      <c r="AD72" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE72" s="41">
+        <v>0.05</v>
+      </c>
+      <c r="AG72" s="78">
+        <v>40.854999999999997</v>
+      </c>
+      <c r="AH72" s="81">
+        <v>1.0999973075576857</v>
+      </c>
+      <c r="AI72" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ72" s="41">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="74" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB74" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AC74" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="AD74" s="8"/>
+      <c r="AE74" s="9" t="s">
+        <v>3</v>
+      </c>
+      <c r="AG74" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="AH74" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="AI74" s="8"/>
+      <c r="AJ74" s="10" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="75" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB75" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AC75" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AD75" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AE75" s="21" t="s">
+        <v>11</v>
+      </c>
+      <c r="AG75" s="75" t="s">
+        <v>25</v>
+      </c>
+      <c r="AH75" s="76" t="s">
+        <v>9</v>
+      </c>
+      <c r="AI75" s="77" t="s">
+        <v>10</v>
+      </c>
+      <c r="AJ75" s="21" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="76" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB76" s="27">
+        <v>197.90819999999999</v>
+      </c>
+      <c r="AC76" s="79">
+        <v>1</v>
+      </c>
+      <c r="AD76" s="29">
+        <v>0</v>
+      </c>
+      <c r="AE76" s="30">
+        <v>0</v>
+      </c>
+      <c r="AG76" s="27">
+        <v>203.4</v>
+      </c>
+      <c r="AH76" s="28">
+        <v>1</v>
+      </c>
+      <c r="AI76" s="29">
+        <v>0</v>
+      </c>
+      <c r="AJ76" s="30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB77" s="31">
+        <v>198.45738</v>
+      </c>
+      <c r="AC77" s="79">
+        <v>1.0027749229188079</v>
+      </c>
+      <c r="AD77" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AE77" s="34">
+        <v>5.000000000000001E-3</v>
+      </c>
+      <c r="AG77" s="31">
+        <v>203.56</v>
+      </c>
+      <c r="AH77" s="32">
+        <v>1.0007866273352999</v>
+      </c>
+      <c r="AI77" s="33">
+        <v>0.1</v>
+      </c>
+      <c r="AJ77" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+    </row>
+    <row r="78" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB78" s="31">
+        <v>199.00656000000001</v>
+      </c>
+      <c r="AC78" s="79">
+        <v>1.0055498458376158</v>
+      </c>
+      <c r="AD78" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AE78" s="34">
+        <v>1.0000000000000002E-2</v>
+      </c>
+      <c r="AG78" s="31">
+        <v>203.72</v>
+      </c>
+      <c r="AH78" s="32">
+        <v>1.0015732546705998</v>
+      </c>
+      <c r="AI78" s="33">
+        <v>0.2</v>
+      </c>
+      <c r="AJ78" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+    </row>
+    <row r="79" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB79" s="31">
+        <v>199.55574000000001</v>
+      </c>
+      <c r="AC79" s="79">
+        <v>1.0083247687564236</v>
+      </c>
+      <c r="AD79" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AE79" s="34">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="AG79" s="31">
+        <v>203.88</v>
+      </c>
+      <c r="AH79" s="32">
+        <v>1.0023598820058996</v>
+      </c>
+      <c r="AI79" s="33">
+        <v>0.3</v>
+      </c>
+      <c r="AJ79" s="34">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="80" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB80" s="31">
+        <v>200.10492000000002</v>
+      </c>
+      <c r="AC80" s="79">
+        <v>1.0110996916752313</v>
+      </c>
+      <c r="AD80" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AE80" s="34">
+        <v>2.0000000000000004E-2</v>
+      </c>
+      <c r="AG80" s="31">
+        <v>204.04</v>
+      </c>
+      <c r="AH80" s="32">
+        <v>1.0031465093411995</v>
+      </c>
+      <c r="AI80" s="33">
+        <v>0.4</v>
+      </c>
+      <c r="AJ80" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+    </row>
+    <row r="81" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB81" s="31">
+        <v>200.65410000000003</v>
+      </c>
+      <c r="AC81" s="79">
+        <v>1.0138746145940392</v>
+      </c>
+      <c r="AD81" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AE81" s="34">
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="AG81" s="31">
+        <v>204.2</v>
+      </c>
+      <c r="AH81" s="32">
+        <v>1.0039331366764994</v>
+      </c>
+      <c r="AI81" s="33">
+        <v>0.5</v>
+      </c>
+      <c r="AJ81" s="34">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="82" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB82" s="31">
+        <v>201.20328000000003</v>
+      </c>
+      <c r="AC82" s="79">
+        <v>1.016649537512847</v>
+      </c>
+      <c r="AD82" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AE82" s="34">
+        <v>0.03</v>
+      </c>
+      <c r="AG82" s="31">
+        <v>204.35999999999999</v>
+      </c>
+      <c r="AH82" s="32">
+        <v>1.0047197640117993</v>
+      </c>
+      <c r="AI82" s="33">
+        <v>0.6</v>
+      </c>
+      <c r="AJ82" s="34">
+        <v>0.06</v>
+      </c>
+    </row>
+    <row r="83" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB83" s="31">
+        <v>201.75246000000004</v>
+      </c>
+      <c r="AC83" s="79">
+        <v>1.0194244604316549</v>
+      </c>
+      <c r="AD83" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AE83" s="34">
+        <v>3.4999999999999996E-2</v>
+      </c>
+      <c r="AG83" s="31">
+        <v>204.51999999999998</v>
+      </c>
+      <c r="AH83" s="32">
+        <v>1.0055063913470992</v>
+      </c>
+      <c r="AI83" s="33">
+        <v>0.7</v>
+      </c>
+      <c r="AJ83" s="34">
+        <v>6.9999999999999993E-2</v>
+      </c>
+    </row>
+    <row r="84" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB84" s="31">
+        <v>202.30164000000005</v>
+      </c>
+      <c r="AC84" s="79">
+        <v>1.0221993833504628</v>
+      </c>
+      <c r="AD84" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AE84" s="34">
+        <v>4.0000000000000008E-2</v>
+      </c>
+      <c r="AG84" s="31">
+        <v>204.67999999999998</v>
+      </c>
+      <c r="AH84" s="32">
+        <v>1.0062930186823991</v>
+      </c>
+      <c r="AI84" s="33">
+        <v>0.8</v>
+      </c>
+      <c r="AJ84" s="34">
+        <v>8.0000000000000016E-2</v>
+      </c>
+    </row>
+    <row r="85" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB85" s="31">
+        <v>202.85082000000006</v>
+      </c>
+      <c r="AC85" s="79">
+        <v>1.0249743062692707</v>
+      </c>
+      <c r="AD85" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AE85" s="34">
+        <v>4.5000000000000005E-2</v>
+      </c>
+      <c r="AG85" s="31">
+        <v>204.83999999999997</v>
+      </c>
+      <c r="AH85" s="32">
+        <v>1.0070796460176989</v>
+      </c>
+      <c r="AI85" s="33">
+        <v>0.9</v>
+      </c>
+      <c r="AJ85" s="34">
+        <v>9.0000000000000011E-2</v>
+      </c>
+    </row>
+    <row r="86" spans="28:36" x14ac:dyDescent="0.25">
+      <c r="AB86" s="78">
+        <v>203.4</v>
+      </c>
+      <c r="AC86" s="79">
+        <v>1.0277492291880781</v>
+      </c>
+      <c r="AD86" s="41">
+        <v>1</v>
+      </c>
+      <c r="AE86" s="41">
+        <v>0.05</v>
+      </c>
+      <c r="AG86" s="78">
+        <v>205</v>
+      </c>
+      <c r="AH86" s="81">
+        <v>1.0078662733529991</v>
+      </c>
+      <c r="AI86" s="41">
+        <v>1</v>
+      </c>
+      <c r="AJ86" s="41">
+        <v>0.1</v>
       </c>
     </row>
   </sheetData>
@@ -13569,7 +16277,7 @@
     <row r="15" spans="1:43" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:43" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43"/>
-      <c r="B16" s="155" t="s">
+      <c r="B16" s="147" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="44" t="s">
@@ -14464,7 +17172,7 @@
     </row>
     <row r="25" spans="1:35" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43"/>
-      <c r="B25" s="155"/>
+      <c r="B25" s="147"/>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
@@ -15124,8 +17832,8 @@
       </c>
     </row>
     <row r="34" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="C34" s="162"/>
-      <c r="D34" s="162"/>
+      <c r="C34" s="154"/>
+      <c r="D34" s="154"/>
       <c r="L34" s="31">
         <f t="shared" si="41"/>
         <v>281.80855199999996</v>
@@ -19967,7 +22675,7 @@
     <row r="15" spans="1:43" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:43" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43"/>
-      <c r="B16" s="155" t="s">
+      <c r="B16" s="147" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="44" t="s">
@@ -20862,7 +23570,7 @@
     </row>
     <row r="25" spans="1:35" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43"/>
-      <c r="B25" s="155"/>
+      <c r="B25" s="147"/>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
@@ -21522,8 +24230,8 @@
       </c>
     </row>
     <row r="34" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="C34" s="162"/>
-      <c r="D34" s="162"/>
+      <c r="C34" s="154"/>
+      <c r="D34" s="154"/>
       <c r="L34" s="31">
         <f t="shared" si="41"/>
         <v>281.80855199999996</v>
@@ -26367,7 +29075,7 @@
     <row r="15" spans="1:43" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="16" spans="1:43" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="43"/>
-      <c r="B16" s="155" t="s">
+      <c r="B16" s="147" t="s">
         <v>21</v>
       </c>
       <c r="C16" s="44" t="s">
@@ -26977,27 +29685,27 @@
       <c r="A22" s="63" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="163" t="str">
+      <c r="B22" s="155" t="str">
         <f>$B$8</f>
         <v>NSV Prem+ Total</v>
       </c>
-      <c r="C22" s="164">
-        <v>0</v>
-      </c>
-      <c r="D22" s="164">
-        <v>0</v>
-      </c>
-      <c r="E22" s="164">
-        <v>0</v>
-      </c>
-      <c r="F22" s="165">
-        <v>0</v>
-      </c>
-      <c r="G22" s="166">
+      <c r="C22" s="156">
+        <v>0</v>
+      </c>
+      <c r="D22" s="156">
+        <v>0</v>
+      </c>
+      <c r="E22" s="156">
+        <v>0</v>
+      </c>
+      <c r="F22" s="157">
+        <v>0</v>
+      </c>
+      <c r="G22" s="158">
         <f t="shared" si="16"/>
         <v>0</v>
       </c>
-      <c r="H22" s="167"/>
+      <c r="H22" s="159"/>
       <c r="I22" s="62">
         <v>0</v>
       </c>
@@ -27262,7 +29970,7 @@
     </row>
     <row r="25" spans="1:35" ht="18.600000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="43"/>
-      <c r="B25" s="155"/>
+      <c r="B25" s="147"/>
       <c r="C25" s="44"/>
       <c r="D25" s="44"/>
       <c r="E25" s="44"/>
@@ -27922,8 +30630,8 @@
       </c>
     </row>
     <row r="34" spans="3:35" x14ac:dyDescent="0.25">
-      <c r="C34" s="162"/>
-      <c r="D34" s="162"/>
+      <c r="C34" s="154"/>
+      <c r="D34" s="154"/>
       <c r="L34" s="31">
         <f t="shared" si="41"/>
         <v>281.80855199999996</v>

</xml_diff>